<commit_message>
#1 Pull down resistors added on unused inputs, center RCA jack color changed, BOM and PDF updated
</commit_message>
<xml_diff>
--- a/Design-Files/Audio-Switcher-v1.2/BOM/Client_BOM-Audio-Switcher-v1.2.xlsx
+++ b/Design-Files/Audio-Switcher-v1.2/BOM/Client_BOM-Audio-Switcher-v1.2.xlsx
@@ -1,20 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\bradfairman-audioswitcher-hw\Design-Files\Audio-Switcher-v1.2\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC2187C4-B66F-4578-8A78-8FDE8BEAB752}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -96,9 +108,6 @@
     <t>C9</t>
   </si>
   <si>
-    <t>C12, C13, C16, C17, C18, C19, C20, C21, C22, C23, C24, C26, C27, C28, C30, C31, C42, C43, C44, C45</t>
-  </si>
-  <si>
     <t>C14, C15</t>
   </si>
   <si>
@@ -123,15 +132,9 @@
     <t>J4</t>
   </si>
   <si>
-    <t>J7, J8, J17, J20, J22</t>
-  </si>
-  <si>
     <t>J11</t>
   </si>
   <si>
-    <t>J13, J15, J18, J19, J21, J23</t>
-  </si>
-  <si>
     <t>L1, L4</t>
   </si>
   <si>
@@ -150,9 +153,6 @@
     <t>R3, R11, R19, R24, R26, R28, R29, R30, R31, R33</t>
   </si>
   <si>
-    <t>R4, R5, R16, R17, R20, R25, R32, R40, R41, R42, R43, R44, R45</t>
-  </si>
-  <si>
     <t>R6, R10, R13, R18, R21, R27, R36, R39</t>
   </si>
   <si>
@@ -592,12 +592,24 @@
   </si>
   <si>
     <t>GRM158R61A226ME15D</t>
+  </si>
+  <si>
+    <t>R4, R5, R16, R17, R20, R25, R32, R40, R41, R42, R43, R44, R45, R47, R56</t>
+  </si>
+  <si>
+    <t>C12, C13, C19, C21, C22, C23, C24, C26, C27, C28, C30, C31, C42, C43, C44, C45</t>
+  </si>
+  <si>
+    <t>J8, J17, J20, J22</t>
+  </si>
+  <si>
+    <t>J7, J13, J15, J18, J19, J21, J23</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1082,7 +1094,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1124,25 +1136,25 @@
         <v>16</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1158,19 +1170,19 @@
         <v>17</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="J3" s="7">
         <v>1</v>
@@ -1190,19 +1202,19 @@
         <v>18</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="J4" s="9">
         <v>2</v>
@@ -1222,19 +1234,19 @@
         <v>19</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="J5" s="7">
         <v>10</v>
@@ -1254,19 +1266,19 @@
         <v>20</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -1286,19 +1298,19 @@
         <v>21</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="J7" s="7">
         <v>4</v>
@@ -1318,19 +1330,19 @@
         <v>22</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="J8" s="9">
         <v>2</v>
@@ -1350,19 +1362,19 @@
         <v>23</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1382,19 +1394,19 @@
         <v>24</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
@@ -1411,25 +1423,25 @@
         <v>2</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>25</v>
+        <v>188</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="J11" s="7">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="K11" s="7"/>
     </row>
@@ -1443,22 +1455,22 @@
         <v>2</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="J12" s="9">
         <v>2</v>
@@ -1475,22 +1487,22 @@
         <v>2</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
@@ -1507,22 +1519,22 @@
         <v>3</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1539,22 +1551,22 @@
         <v>4</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -1571,22 +1583,22 @@
         <v>5</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="I16" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
@@ -1603,22 +1615,22 @@
         <v>6</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -1635,22 +1647,22 @@
         <v>7</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J18" s="9">
         <v>8</v>
@@ -1667,22 +1679,22 @@
         <v>7</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
@@ -1699,25 +1711,25 @@
         <v>7</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>34</v>
+        <v>189</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J20" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K20" s="9"/>
     </row>
@@ -1731,22 +1743,22 @@
         <v>8</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J21" s="7">
         <v>1</v>
@@ -1763,25 +1775,25 @@
         <v>7</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>36</v>
+        <v>190</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J22" s="9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K22" s="9"/>
     </row>
@@ -1795,22 +1807,22 @@
         <v>9</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="J23" s="7">
         <v>2</v>
@@ -1827,22 +1839,22 @@
         <v>9</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J24" s="9">
         <v>2</v>
@@ -1859,22 +1871,22 @@
         <v>10</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J25" s="7">
         <v>5</v>
@@ -1891,22 +1903,22 @@
         <v>11</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J26" s="9">
         <v>8</v>
@@ -1923,22 +1935,22 @@
         <v>12</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="J27" s="7">
         <v>4</v>
@@ -1955,22 +1967,22 @@
         <v>12</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="J28" s="9">
         <v>10</v>
@@ -1987,25 +1999,25 @@
         <v>12</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>43</v>
+        <v>187</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="J29" s="7">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K29" s="7"/>
     </row>
@@ -2019,22 +2031,22 @@
         <v>12</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="J30" s="9">
         <v>8</v>
@@ -2051,22 +2063,22 @@
         <v>12</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J31" s="7">
         <v>5</v>
@@ -2083,22 +2095,22 @@
         <v>12</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="J32" s="9">
         <v>14</v>
@@ -2115,22 +2127,22 @@
         <v>13</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2147,22 +2159,22 @@
         <v>14</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="I34" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
@@ -2179,22 +2191,22 @@
         <v>14</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
@@ -2211,22 +2223,22 @@
         <v>14</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="I36" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J36" s="9">
         <v>1</v>
@@ -2243,22 +2255,22 @@
         <v>14</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J37" s="7">
         <v>1</v>
@@ -2275,22 +2287,22 @@
         <v>14</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="I38" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J38" s="9">
         <v>1</v>
@@ -2307,22 +2319,22 @@
         <v>15</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="J39" s="7">
         <v>1</v>

</xml_diff>